<commit_message>
first new ARB test
</commit_message>
<xml_diff>
--- a/docs/rail_calculator.xlsx
+++ b/docs/rail_calculator.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mods\unpacked\un1corn_qlourie_astral_r\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\un1corn\UserSpace\Games\Steam_Library\common\BeamNG_Userdata\current\mods\unpacked\un1corn_qlourie_astral_r\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36E638D6-745C-4F90-BA54-387632E13E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5819EA1-07A8-4567-8637-ED93449F6C68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,109 +36,115 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>X</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Y</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Z</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>P1</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>P2</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>P3X</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>P3Y</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>P3Z</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Length</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>A</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Rear Top</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Front Top</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Front Gravel Caster</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Rear Gravel Caster</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Rear Gravel Bottom</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Front Gravel Bottom</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Rear Arm</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Front Arm</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Rear Tarmac Bottom</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Rear Tarmac Caster</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Front Tarmac Bottom</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Front Tarmac Caster</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Rear RX Caster</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Front RX Caster</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Rail calculator</t>
+  </si>
+  <si>
+    <t>坐标与长度单位：m。黄色单元格为手动输入。</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -156,22 +162,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="等线"/>
       <family val="2"/>
@@ -204,11 +194,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF195DB1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF667B91"/>
       <name val="Arial"/>
     </font>
@@ -278,6 +263,8 @@
       <sz val="10"/>
       <color rgb="FF667B91"/>
       <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
@@ -290,7 +277,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="25">
+  <fills count="23">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -310,12 +297,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
@@ -331,61 +312,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDF2F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDF2F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEDF2F7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEDF2F7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF5F7FA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF5F7FA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF5F7FA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
@@ -409,33 +390,13 @@
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="22">
+  <borders count="20">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -474,6 +435,20 @@
       <left/>
       <right/>
       <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color rgb="FFDCE4EB"/>
       </bottom>
@@ -483,20 +458,6 @@
       <left/>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="thin">
         <color rgb="FFDCE4EB"/>
       </bottom>
@@ -569,15 +530,6 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="thin">
-        <color rgb="FFDCE4EB"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -605,86 +557,77 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="2" applyBorder="1" applyAlignment="1" applyFont="1" applyFill="1">
-      <alignment vertical="center" horizontal="left" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="2" applyBorder="1" applyAlignment="1" applyFont="1" applyFill="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="2" applyBorder="1" applyAlignment="1" applyFont="1" applyFill="1">
-      <alignment vertical="center" horizontal="left" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="right" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="6" xfId="2" applyBorder="1" applyAlignment="1" applyFont="1" applyFill="1">
-      <alignment vertical="center" horizontal="left" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="7" xfId="1" applyAlignment="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="8" xfId="1" applyAlignment="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center" horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="right" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="10" xfId="2" applyBorder="1" applyAlignment="1" applyFont="1" applyFill="1">
-      <alignment vertical="center" horizontal="right" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="11" xfId="2" applyBorder="1" applyAlignment="1" applyFont="1" applyFill="1">
-      <alignment vertical="center" horizontal="right" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="12" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1" applyFont="1">
-      <alignment vertical="center" horizontal="right" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="16" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="right" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center" horizontal="left" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="right" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center" horizontal="left" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="right" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="0"/>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="16" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="40% - 着色 1" xfId="2" builtinId="31"/>
-    <cellStyle name="差" xfId="1" builtinId="27"/>
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="40% - Accent1" xfId="2" builtinId="31"/>
+    <cellStyle name="Bad" xfId="1" builtinId="27"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -962,363 +905,355 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H24"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31" customWidth="1"/>
-    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="16" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="31" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="6" max="8" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3" ht="35" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Rail calculator</t>
-        </is>
-      </c>
-      <c r="B1" s="8" t="s">
+    <row r="1" spans="1:8" ht="35.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3" ht="30" customHeight="1">
-      <c r="A2" s="9" t="s">
+    <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="15">
+        <v>0.752</v>
+      </c>
+      <c r="C2" s="15">
+        <v>-1.2949999999999999</v>
+      </c>
+      <c r="D2" s="15">
+        <v>2.1000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="15">
+        <v>0.27200000000000002</v>
+      </c>
+      <c r="C3" s="15">
+        <v>-0.97499999999999998</v>
+      </c>
+      <c r="D3" s="15">
+        <v>0.105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="6">
+        <f>SQRT((B3-B2)^2+(C3-C2)^2+(D3-D2)^2)</f>
+        <v>0.58297169742621291</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="7">
+        <v>0.47899999999999998</v>
+      </c>
+      <c r="C5" s="8">
+        <f>((B5-B3)/(B3-B2))*(C3-C2)+C3</f>
+        <v>-1.113</v>
+      </c>
+      <c r="D5" s="8">
+        <f>((B5-B3)/(B3-B2))*(D3-D2)+D3</f>
+        <v>6.8775000000000003E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="9">
+        <f>((C6-C3)/(C3-C2))*(B3-B2)+B3</f>
+        <v>-1.1905000000000001</v>
+      </c>
+      <c r="C6" s="10">
+        <v>0</v>
+      </c>
+      <c r="D6" s="9">
+        <f>((C6-C3)/(C3-C2))*(D3-D2)+D3</f>
+        <v>0.36093749999999997</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="8">
+        <f>((D7-D3)/(D3-D2))*(B3-B2)+B3</f>
+        <v>-0.47085714285714297</v>
+      </c>
+      <c r="C7" s="8">
+        <f>((D7-D3)/(D3-D2))*(C3-C2)+C3</f>
+        <v>-0.47976190476190472</v>
+      </c>
+      <c r="D7" s="11">
+        <v>0.23499999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" s="18"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+    </row>
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="13">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="C9" s="13">
+        <v>1.337</v>
+      </c>
+      <c r="D9" s="13">
+        <v>0.79700000000000004</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="15">
         <v>0.222</v>
       </c>
-      <c r="C2" s="10">
+      <c r="C10" s="15">
         <v>1.333</v>
       </c>
-      <c r="D2" s="10">
+      <c r="D10" s="15">
         <v>0.108</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3" ht="30" customHeight="1">
-      <c r="A3" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="10">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="13">
+        <v>0.57640000000000002</v>
+      </c>
+      <c r="C11" s="13">
+        <v>1.355</v>
+      </c>
+      <c r="D11" s="13">
+        <v>1.41E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="15">
         <v>0.747</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C12" s="15">
         <v>1.3009999999999999</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D12" s="15">
         <v>-6.3E-2</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3" ht="32" customHeight="1">
-      <c r="A4" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="13">
-        <f>SQRT((B3-B2)^2+(C3-C2)^2+(D3-D2)^2)</f>
-        <v>0.55307323204074887</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3" ht="30" customHeight="1">
-      <c r="A5" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="14">
-        <v>0.438</v>
-      </c>
-      <c r="C5" s="15">
-        <f>((B5-B3)/(B3-B2))*(C3-C2)+C3</f>
-        <v>1.3198342857142857</v>
-      </c>
-      <c r="D5" s="15">
-        <f>((B5-B3)/(B3-B2))*(D3-D2)+D3</f>
-        <v>3.7645714285714268E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3" ht="30" customHeight="1">
-      <c r="A6" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="16">
-        <f>((C6-C3)/(C3-C2))*(B3-B2)+B3</f>
-        <v>22.091531249999981</v>
-      </c>
-      <c r="C6" s="17">
-        <v>0</v>
-      </c>
-      <c r="D6" s="16">
-        <f>((C6-C3)/(C3-C2))*(D3-D2)+D3</f>
-        <v>-7.0152187499999927</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3" ht="30" customHeight="1">
-      <c r="A7" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="15">
-        <f>((D7-D3)/(D3-D2))*(B3-B2)+B3</f>
-        <v>-0.16791228070175446</v>
-      </c>
-      <c r="C7" s="15">
-        <f>((D7-D3)/(D3-D2))*(C3-C2)+C3</f>
-        <v>1.356766081871345</v>
-      </c>
-      <c r="D7" s="18">
-        <v>0.23499999999999999</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="25"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="25"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3" ht="30" customHeight="1">
-      <c r="A9" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="20">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="C9" s="20">
-        <v>1.337</v>
-      </c>
-      <c r="D9" s="20">
-        <v>0.79700000000000004</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3" ht="30" customHeight="1">
-      <c r="A10" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="22">
-        <v>0.222</v>
-      </c>
-      <c r="C10" s="22">
-        <v>1.333</v>
-      </c>
-      <c r="D10" s="22">
-        <v>0.108</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3" ht="30" customHeight="1">
-      <c r="A11" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="20">
-        <v>0.57640000000000002</v>
-      </c>
-      <c r="C11" s="20">
-        <v>1.355</v>
-      </c>
-      <c r="D11" s="20">
-        <v>1.41E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3" ht="30" customHeight="1">
-      <c r="A12" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="22">
+      <c r="E12" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="13">
         <v>0.747</v>
       </c>
-      <c r="C12" s="22">
+      <c r="G12" s="13">
         <v>1.3009999999999999</v>
       </c>
-      <c r="D12" s="22">
+      <c r="H12" s="13">
         <v>-6.3E-2</v>
       </c>
-      <c r="E12" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="F12" s="20">
+    </row>
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="13">
+        <v>0.56769999999999998</v>
+      </c>
+      <c r="C13" s="13">
+        <v>1.351</v>
+      </c>
+      <c r="D13" s="13">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="15">
+        <v>0.749</v>
+      </c>
+      <c r="C14" s="15">
+        <v>1.341</v>
+      </c>
+      <c r="D14" s="15">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15" s="16"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+    </row>
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" s="13">
+        <v>0.58099999999999996</v>
+      </c>
+      <c r="C16" s="13">
+        <v>-1.22</v>
+      </c>
+      <c r="D16" s="13">
+        <v>0.81499999999999995</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="15">
+        <v>0.27200000000000002</v>
+      </c>
+      <c r="C17" s="15">
+        <v>-0.97499999999999998</v>
+      </c>
+      <c r="D17" s="15">
+        <v>0.105</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" s="13">
+        <v>0.62270000000000003</v>
+      </c>
+      <c r="C18" s="13">
+        <v>-1.3589</v>
+      </c>
+      <c r="D18" s="13">
+        <v>5.0700000000000002E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="15">
         <v>0.747</v>
       </c>
-      <c r="G12" s="20">
-        <v>1.3009999999999999</v>
-      </c>
-      <c r="H12" s="20">
+      <c r="C19" s="15">
+        <v>-1.3</v>
+      </c>
+      <c r="D19" s="15">
+        <v>-5.2999999999999999E-2</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F19" s="13">
+        <v>0.747</v>
+      </c>
+      <c r="G19" s="13">
+        <v>-1.3</v>
+      </c>
+      <c r="H19" s="13">
         <v>-6.3E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3" ht="30" customHeight="1">
-      <c r="A13" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="20">
-        <v>0.56769999999999998</v>
-      </c>
-      <c r="C13" s="20">
-        <v>1.351</v>
-      </c>
-      <c r="D13" s="20">
-        <v>0.17</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3" ht="30" customHeight="1">
-      <c r="A14" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="22">
-        <v>0.749</v>
-      </c>
-      <c r="C14" s="22">
-        <v>1.341</v>
-      </c>
-      <c r="D14" s="22">
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="23"/>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3" ht="30" customHeight="1">
-      <c r="A16" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="B16" s="20">
-        <v>0.58099999999999996</v>
-      </c>
-      <c r="C16" s="20">
-        <v>-1.22</v>
-      </c>
-      <c r="D16" s="20">
-        <v>0.81499999999999995</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="21" t="s">
-        <v>17</v>
-      </c>
-      <c r="B17" s="22">
-        <v>0.27200000000000002</v>
-      </c>
-      <c r="C17" s="22">
-        <v>-0.97499999999999998</v>
-      </c>
-      <c r="D17" s="22">
-        <v>0.105</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3" ht="30" customHeight="1">
-      <c r="A18" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B18" s="20">
-        <v>0.62270000000000003</v>
-      </c>
-      <c r="C18" s="20">
-        <v>-1.3589</v>
-      </c>
-      <c r="D18" s="20">
-        <v>5.0700000000000002E-2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3" ht="30" customHeight="1">
-      <c r="A19" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B19" s="22">
-        <v>0.747</v>
-      </c>
-      <c r="C19" s="22">
-        <v>-1.3</v>
-      </c>
-      <c r="D19" s="22">
-        <v>-5.2999999999999999E-2</v>
-      </c>
-      <c r="E19" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="F19" s="20">
-        <v>0.747</v>
-      </c>
-      <c r="G19" s="20">
-        <v>-1.3</v>
-      </c>
-      <c r="H19" s="20">
-        <v>-6.3E-2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="19" t="s">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="20">
+      <c r="B20" s="13">
         <v>0.61099999999999999</v>
       </c>
-      <c r="C20" s="20">
+      <c r="C20" s="13">
         <v>-1.333</v>
       </c>
-      <c r="D20" s="20">
+      <c r="D20" s="13">
         <v>0.20300000000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3" ht="30" customHeight="1">
-      <c r="A21" s="21" t="s">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="22">
+      <c r="B21" s="15">
         <v>0.752</v>
       </c>
-      <c r="C21" s="22">
+      <c r="C21" s="15">
         <v>-1.2949999999999999</v>
       </c>
-      <c r="D21" s="22">
+      <c r="D21" s="15">
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="25"/>
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
-    </row>
-    <row r="23" ht="28" customHeight="1">
-      <c r="A23" t="inlineStr" s="24">
-        <is>
-          <t>坐标与长度单位：m。黄色单元格为手动输入。</t>
-        </is>
-      </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="26"/>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" s="18"/>
+      <c r="B22" s="18"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="18"/>
+    </row>
+    <row r="23" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
+      <c r="G23" s="19"/>
+      <c r="H23" s="19"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>